<commit_message>
feat: apply specialist QA revisions (12 QAs), optimize BGE-M3 CUDA/TF32 and summary merge
</commit_message>
<xml_diff>
--- a/Resultados/Resultados_TCC_3_Abas_GoogleSheets.xlsx
+++ b/Resultados/Resultados_TCC_3_Abas_GoogleSheets.xlsx
@@ -946,42 +946,168 @@
     <row r="19" ht="44" customHeight="1">
       <c r="A19" t="inlineStr" s="3">
         <is>
-          <t>SEMANTIC (SemanticChunker BGE-M3)</t>
+          <t>SEMANTIC p40 (SemanticChunker BGE-M3)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="3">
         <is>
-          <t>Threshold = Percentil 60 (p60) da distância de cosseno</t>
+          <t>Threshold = Percentil 40 (p40) da distância de cosseno</t>
         </is>
       </c>
       <c r="C19" s="3">
-        <v>781</v>
+        <v>1165</v>
       </c>
       <c r="D19" s="3">
-        <v>385.5</v>
+        <v>258.4</v>
       </c>
       <c r="E19" s="3">
         <v>9.78</v>
       </c>
       <c r="F19" s="3">
+        <v>169.0837</v>
+      </c>
+      <c r="G19" t="inlineStr" s="3">
+        <is>
+          <t>2.692x mais lento que Fixed (primeira passagem BGE-M3)</t>
+        </is>
+      </c>
+      <c r="H19" s="3">
+        <v>142.34</v>
+      </c>
+      <c r="I19" t="inlineStr" s="3">
+        <is>
+          <t>311.42 s (~5 min 11 s)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr" s="3">
+        <is>
+          <t>Mais sensível a mudanças sutis de assunto: corta em 60% das transições entre sentenças, gerando 1.165 micro-chunks (~258 chars em média).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" t="inlineStr" s="3">
+        <is>
+          <t>SEMANTIC p50 (SemanticChunker BGE-M3)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="3">
+        <is>
+          <t>Threshold = Percentil 50 (p50 — Mediana) da distância de cosseno</t>
+        </is>
+      </c>
+      <c r="C20" s="3">
+        <v>970</v>
+      </c>
+      <c r="D20" s="3">
+        <v>310.4</v>
+      </c>
+      <c r="E20" s="3">
+        <v>9.78</v>
+      </c>
+      <c r="F20" s="4">
+        <v>0.0258</v>
+      </c>
+      <c r="G20" t="inlineStr" s="3">
+        <is>
+          <t>0.026s com cache de sentenças (~170s sem cache)</t>
+        </is>
+      </c>
+      <c r="H20" s="3">
+        <v>139.0</v>
+      </c>
+      <c r="I20" t="inlineStr" s="3">
+        <is>
+          <t>139.03 s (com cache de embeddings de sentenças)</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr" s="3">
+        <is>
+          <t>Corta exatamente na mediana das distâncias de cosseno entre sentenças adjacentes (970 chunks de ~310 chars). Obteve o RECORDE GERAL de Answer Correctness (0.2731) e Answer Relevancy (0.3793) em K=3!</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="A21" t="inlineStr" s="3">
+        <is>
+          <t>SEMANTIC p60 (SemanticChunker BGE-M3)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="3">
+        <is>
+          <t>Threshold = Percentil 60 (p60) da distância de cosseno</t>
+        </is>
+      </c>
+      <c r="C21" s="3">
+        <v>781</v>
+      </c>
+      <c r="D21" s="3">
+        <v>385.5</v>
+      </c>
+      <c r="E21" s="3">
+        <v>9.78</v>
+      </c>
+      <c r="F21" s="3">
         <v>170.3863</v>
       </c>
-      <c r="G19" t="inlineStr" s="3">
+      <c r="G21" t="inlineStr" s="3">
         <is>
           <t>2.713x mais lento que Fixed (~2 min 50 s só para chunkar!)</t>
         </is>
       </c>
-      <c r="H19" s="3">
+      <c r="H21" s="3">
         <v>131.69</v>
       </c>
-      <c r="I19" t="inlineStr" s="3">
+      <c r="I21" t="inlineStr" s="3">
         <is>
           <t>302.07 s (~5 min 02 s — 2.4x mais lento no total)</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr" s="3">
-        <is>
-          <t>Exige calcular embeddings BAAI/bge-m3 em CPU para TODAS as 1.981 sentenças dos 10 PDFs durante a etapa de chunking para medir a distância de cosseno entre sentenças adjacentes, e depois re-embeda os 781 chunks resultantes para indexar no Chroma.</t>
+      <c r="J21" t="inlineStr" s="3">
+        <is>
+          <t>Exige calcular embeddings BAAI/bge-m3 para TODAS as 1.981 sentenças dos 10 PDFs durante a etapa de chunking para medir a distância de cosseno entre sentenças adjacentes, e depois re-embeda os 781 chunks resultantes para indexar no Chroma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="A22" t="inlineStr" s="3">
+        <is>
+          <t>SEMANTIC p70 (SemanticChunker BGE-M3)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="3">
+        <is>
+          <t>Threshold = Percentil 70 (p70) da distância de cosseno</t>
+        </is>
+      </c>
+      <c r="C22" s="3">
+        <v>590</v>
+      </c>
+      <c r="D22" s="3">
+        <v>510.3</v>
+      </c>
+      <c r="E22" s="3">
+        <v>9.78</v>
+      </c>
+      <c r="F22" s="4">
+        <v>0.0256</v>
+      </c>
+      <c r="G22" t="inlineStr" s="3">
+        <is>
+          <t>0.026s com cache de sentenças (~170s sem cache)</t>
+        </is>
+      </c>
+      <c r="H22" s="3">
+        <v>125.63</v>
+      </c>
+      <c r="I22" t="inlineStr" s="3">
+        <is>
+          <t>125.66 s (com cache de embeddings de sentenças)</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr" s="3">
+        <is>
+          <t>Mais conservador: corta apenas nos 30% maiores saltos semânticos, gerando 590 chunks maiores (~510 chars).</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1349,7 @@
     <row r="5" ht="44" customHeight="1">
       <c r="A5" t="inlineStr" s="3">
         <is>
-          <t>SEMANTIC p60 (K=3)</t>
+          <t>SEMANTIC p40 (K=3)</t>
         </is>
       </c>
       <c r="B5" s="3">
@@ -1231,14 +1357,14 @@
       </c>
       <c r="C5" t="inlineStr" s="3">
         <is>
-          <t>Percentil 60 (p60) | teto 2000 chars/chunk</t>
+          <t>Percentil 40 (p40) | teto 2000 chars/chunk</t>
         </is>
       </c>
       <c r="D5" s="3">
-        <v>781</v>
+        <v>1165</v>
       </c>
       <c r="E5" s="4">
-        <v>0.3702</v>
+        <v>0.4866</v>
       </c>
       <c r="F5" t="inlineStr" s="3">
         <is>
@@ -1246,7 +1372,7 @@
         </is>
       </c>
       <c r="G5" s="4">
-        <v>0.2836</v>
+        <v>0.2655</v>
       </c>
       <c r="H5" t="inlineStr" s="3">
         <is>
@@ -1254,127 +1380,123 @@
         </is>
       </c>
       <c r="I5" s="4">
-        <v>0.2513</v>
+        <v>0.214</v>
       </c>
       <c r="J5" t="inlineStr" s="3">
         <is>
-          <t>28/30</t>
+          <t>29/30</t>
         </is>
       </c>
       <c r="K5" s="4">
-        <v>0.7556</v>
+        <v>0.5306</v>
       </c>
       <c r="L5" s="4">
-        <v>0.5085</v>
+        <v>0.3306</v>
       </c>
       <c r="M5" s="3">
-        <v>170.3863</v>
-      </c>
-      <c r="N5" t="inlineStr" s="3">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr" s="3">
-        <is>
-          <t>—</t>
-        </is>
+        <v>169.0837</v>
+      </c>
+      <c r="N5" s="3">
+        <v>177.26</v>
+      </c>
+      <c r="O5" s="3">
+        <v>4.432</v>
       </c>
       <c r="P5" t="inlineStr" s="3">
         <is>
-          <t>Líder geral em Context Recall (0.5085) no K=3: chunks menores (~385 chars) permitem buscar 3 trechos focados em PDFs distintos, mas pouca informação contextual reduz Faithfulness (0.3702).</t>
+          <t>Maior Faithfulness no K=3 (0.4866): chunks super curtos (~258 chars) evitam alucinação, mas 3 micro-chunks são insuficientes para cobrir perguntas complexas (menor Recall = 0.3306 e Precision = 0.5306).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" t="inlineStr" s="3">
         <is>
-          <t>FIXED (K=5)</t>
+          <t>SEMANTIC p50 (K=3)</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr" s="3">
         <is>
-          <t>512 tokens | overlap 51 | teto 1200 chars/chunk</t>
+          <t>Percentil 50 (p50) | teto 2000 chars/chunk</t>
         </is>
       </c>
       <c r="D6" s="3">
-        <v>207</v>
+        <v>970</v>
       </c>
       <c r="E6" s="4">
-        <v>0.4882</v>
+        <v>0.437</v>
       </c>
       <c r="F6" t="inlineStr" s="3">
         <is>
-          <t>29/30</t>
+          <t>27/30</t>
         </is>
       </c>
       <c r="G6" s="4">
-        <v>0.2608</v>
+        <v>0.3793</v>
       </c>
       <c r="H6" t="inlineStr" s="3">
         <is>
-          <t>29/30</t>
+          <t>30/30</t>
         </is>
       </c>
       <c r="I6" s="4">
-        <v>0.2358</v>
+        <v>0.2731</v>
       </c>
       <c r="J6" t="inlineStr" s="3">
         <is>
-          <t>27/30</t>
+          <t>28/30</t>
         </is>
       </c>
       <c r="K6" s="4">
-        <v>0.8354</v>
+        <v>0.6583</v>
       </c>
       <c r="L6" s="4">
-        <v>0.4307</v>
+        <v>0.3904</v>
       </c>
       <c r="M6" s="4">
-        <v>0.0628</v>
+        <v>0.0258</v>
       </c>
       <c r="N6" s="3">
-        <v>185.89</v>
+        <v>180.0</v>
       </c>
       <c r="O6" s="3">
-        <v>3.457</v>
+        <v>5.091</v>
       </c>
       <c r="P6" t="inlineStr" s="3">
         <is>
-          <t>MAIOR FAITHFULNESS DE TODOS OS TESTES (0.4882, salto de +22% sobre K=3!) e Recall subiu de 0.4093 para 0.4307. Trazer 5 chunks deu suporte factual completo para o Llama-3.1-8B não alucinar.</t>
+          <t>RECORDE GERAL DE ANSWER RELEVANCY (0.3793) E ANSWER CORRECTNESS (0.2731)! O corte na mediana (p50, ~310 chars/chunk) equilibrou perfeitamente foco temático e completude da resposta no K=3.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" t="inlineStr" s="3">
         <is>
-          <t>RECURSIVE (K=5)</t>
+          <t>SEMANTIC p60 (K=3)</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr" s="3">
         <is>
-          <t>512 tokens | overlap 51 | teto 1200 chars/chunk</t>
+          <t>Percentil 60 (p60) | teto 2000 chars/chunk</t>
         </is>
       </c>
       <c r="D7" s="3">
-        <v>213</v>
+        <v>781</v>
       </c>
       <c r="E7" s="4">
-        <v>0.4126</v>
+        <v>0.3702</v>
       </c>
       <c r="F7" t="inlineStr" s="3">
         <is>
-          <t>29/30</t>
+          <t>28/30</t>
         </is>
       </c>
       <c r="G7" s="4">
-        <v>0.3169</v>
+        <v>0.2836</v>
       </c>
       <c r="H7" t="inlineStr" s="3">
         <is>
@@ -1382,7 +1504,7 @@
         </is>
       </c>
       <c r="I7" s="4">
-        <v>0.2475</v>
+        <v>0.2513</v>
       </c>
       <c r="J7" t="inlineStr" s="3">
         <is>
@@ -1390,53 +1512,57 @@
         </is>
       </c>
       <c r="K7" s="4">
-        <v>0.7929</v>
+        <v>0.7556</v>
       </c>
       <c r="L7" s="4">
-        <v>0.4426</v>
-      </c>
-      <c r="M7" s="4">
-        <v>0.2182</v>
-      </c>
-      <c r="N7" s="3">
-        <v>181.37</v>
-      </c>
-      <c r="O7" s="3">
-        <v>4.398</v>
+        <v>0.5085</v>
+      </c>
+      <c r="M7" s="3">
+        <v>170.3863</v>
+      </c>
+      <c r="N7" t="inlineStr" s="3">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr" s="3">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P7" t="inlineStr" s="3">
         <is>
-          <t>MAIOR ANSWER RELEVANCY DE TODOS OS TESTES (0.3169, salto de +46% sobre K=3!) e maior Answer Correctness em K=5 (0.2475, +18% sobre K=3). Com 5 chunks, o Recursive parou de se abster nas perguntas multi-documento!</t>
+          <t>Líder geral em Context Recall (0.5085) no K=3: chunks de ~385 chars permitem buscar 3 trechos focados em PDFs distintos, mas pouca informação contextual reduz Faithfulness (0.3702).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" t="inlineStr" s="3">
         <is>
-          <t>SEMANTIC p60 (K=5)</t>
+          <t>SEMANTIC p70 (K=3)</t>
         </is>
       </c>
       <c r="B8" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C8" t="inlineStr" s="3">
         <is>
-          <t>Percentil 60 (p60) | teto 1200 chars/chunk</t>
+          <t>Percentil 70 (p70) | teto 2000 chars/chunk</t>
         </is>
       </c>
       <c r="D8" s="3">
-        <v>781</v>
+        <v>590</v>
       </c>
       <c r="E8" s="4">
-        <v>0.4652</v>
+        <v>0.4456</v>
       </c>
       <c r="F8" t="inlineStr" s="3">
         <is>
-          <t>27/30</t>
+          <t>28/30</t>
         </is>
       </c>
       <c r="G8" s="4">
-        <v>0.2301</v>
+        <v>0.2637</v>
       </c>
       <c r="H8" t="inlineStr" s="3">
         <is>
@@ -1444,115 +1570,115 @@
         </is>
       </c>
       <c r="I8" s="4">
-        <v>0.2457</v>
+        <v>0.236</v>
       </c>
       <c r="J8" t="inlineStr" s="3">
         <is>
-          <t>27/30</t>
+          <t>29/30</t>
         </is>
       </c>
       <c r="K8" s="4">
-        <v>0.6963</v>
+        <v>0.7556</v>
       </c>
       <c r="L8" s="4">
-        <v>0.4581</v>
-      </c>
-      <c r="M8" s="3">
-        <v>170.3863</v>
+        <v>0.4228</v>
+      </c>
+      <c r="M8" s="4">
+        <v>0.0256</v>
       </c>
       <c r="N8" s="3">
-        <v>177.92</v>
+        <v>175.81</v>
       </c>
       <c r="O8" s="3">
-        <v>4.943</v>
+        <v>4.602</v>
       </c>
       <c r="P8" t="inlineStr" s="3">
         <is>
-          <t>Salto expressivo em Faithfulness (+25.7%, de 0.3702 em K=3 para 0.4652 em K=5) e lidera o Context Recall dentro de K=5 (0.4581), pois 5 micro-chunks semânticos formam um contexto mais completo sem sofrer corte no limite de 1200 chars.</t>
+          <t>Chunks maiores (~510 chars, 590 chunks) mantêm alta Context Precision (0.7556, empatado com p60) e boa Faithfulness (0.4456), mas perdem a precisão cirúrgica do p50 na resposta final.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" t="inlineStr" s="3">
         <is>
-          <t>FIXED (K=7)</t>
+          <t>FIXED (K=5)</t>
         </is>
       </c>
       <c r="B9" s="3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C9" t="inlineStr" s="3">
         <is>
-          <t>512 tokens | overlap 51 | teto 857 chars/chunk (TRUNCADO!)</t>
+          <t>512 tokens | overlap 51 | teto 1200 chars/chunk</t>
         </is>
       </c>
       <c r="D9" s="3">
         <v>207</v>
       </c>
       <c r="E9" s="4">
-        <v>0.2693</v>
+        <v>0.4882</v>
       </c>
       <c r="F9" t="inlineStr" s="3">
         <is>
-          <t>28/30</t>
+          <t>29/30</t>
         </is>
       </c>
       <c r="G9" s="4">
-        <v>0.1678</v>
+        <v>0.2608</v>
       </c>
       <c r="H9" t="inlineStr" s="3">
         <is>
-          <t>30/30</t>
+          <t>29/30</t>
         </is>
       </c>
       <c r="I9" s="4">
-        <v>0.1728</v>
+        <v>0.2358</v>
       </c>
       <c r="J9" t="inlineStr" s="3">
         <is>
-          <t>26/30</t>
+          <t>27/30</t>
         </is>
       </c>
       <c r="K9" s="4">
-        <v>0.7199</v>
+        <v>0.8354</v>
       </c>
       <c r="L9" s="4">
-        <v>0.4022</v>
+        <v>0.4307</v>
       </c>
       <c r="M9" s="4">
         <v>0.0628</v>
       </c>
       <c r="N9" s="3">
-        <v>173.29</v>
+        <v>185.89</v>
       </c>
       <c r="O9" s="3">
-        <v>2.38</v>
+        <v>3.457</v>
       </c>
       <c r="P9" t="inlineStr" s="3">
         <is>
-          <t>Queda acentuada em K=7: como RAG_MAX_CONTEXT_CHARS=6000 divide o orçamento por K (6000 // 7 = 857 chars/chunk), cada chunk Fixed (~1454 chars) perde ~41% do seu texto final! Além disso, mais chunks periféricos diluem a atenção do LLM (Lost in the Middle).</t>
+          <t>MAIOR FAITHFULNESS DE TODOS OS TESTES (0.4882, salto de +22% sobre K=3!) e Recall subiu de 0.4093 para 0.4307. Trazer 5 chunks deu suporte factual completo para o Llama-3.1-8B não alucinar.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" t="inlineStr" s="3">
         <is>
-          <t>RECURSIVE (K=7)</t>
+          <t>RECURSIVE (K=5)</t>
         </is>
       </c>
       <c r="B10" s="3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C10" t="inlineStr" s="3">
         <is>
-          <t>512 tokens | overlap 51 | teto 857 chars/chunk (TRUNCADO!)</t>
+          <t>512 tokens | overlap 51 | teto 1200 chars/chunk</t>
         </is>
       </c>
       <c r="D10" s="3">
         <v>213</v>
       </c>
       <c r="E10" s="4">
-        <v>0.3735</v>
+        <v>0.4126</v>
       </c>
       <c r="F10" t="inlineStr" s="3">
         <is>
@@ -1560,7 +1686,7 @@
         </is>
       </c>
       <c r="G10" s="4">
-        <v>0.1647</v>
+        <v>0.3169</v>
       </c>
       <c r="H10" t="inlineStr" s="3">
         <is>
@@ -1568,61 +1694,61 @@
         </is>
       </c>
       <c r="I10" s="4">
-        <v>0.1653</v>
+        <v>0.2475</v>
       </c>
       <c r="J10" t="inlineStr" s="3">
         <is>
-          <t>27/30</t>
+          <t>28/30</t>
         </is>
       </c>
       <c r="K10" s="4">
-        <v>0.7187</v>
+        <v>0.7929</v>
       </c>
       <c r="L10" s="4">
-        <v>0.4961</v>
+        <v>0.4426</v>
       </c>
       <c r="M10" s="4">
         <v>0.2182</v>
       </c>
       <c r="N10" s="3">
-        <v>175.61</v>
+        <v>181.37</v>
       </c>
       <c r="O10" s="3">
-        <v>3.127</v>
+        <v>4.398</v>
       </c>
       <c r="P10" t="inlineStr" s="3">
         <is>
-          <t>O Context Recall subiu para 0.4961 (mais trechos do gabarito entraram nos 7 chunks), mas a qualidade da resposta (Relevancy 0.1647 / Correctness 0.1653) caiu pelo truncamento de 857 chars/chunk no gerador e pelo excesso de ruído no prompt.</t>
+          <t>MAIOR ANSWER RELEVANCY DE TODOS OS TESTES (0.3169, salto de +46% sobre K=3!) e maior Answer Correctness em K=5 (0.2475, +18% sobre K=3). Com 5 chunks, o Recursive parou de se abster nas perguntas multi-documento!</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" t="inlineStr" s="3">
         <is>
-          <t>SEMANTIC p60 (K=7)</t>
+          <t>SEMANTIC p60 (K=5)</t>
         </is>
       </c>
       <c r="B11" s="3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C11" t="inlineStr" s="3">
         <is>
-          <t>Percentil 60 (p60) | teto 857 chars/chunk</t>
+          <t>Percentil 60 (p60) | teto 1200 chars/chunk</t>
         </is>
       </c>
       <c r="D11" s="3">
         <v>781</v>
       </c>
       <c r="E11" s="4">
-        <v>0.3481</v>
+        <v>0.4652</v>
       </c>
       <c r="F11" t="inlineStr" s="3">
         <is>
-          <t>26/30</t>
+          <t>27/30</t>
         </is>
       </c>
       <c r="G11" s="4">
-        <v>0.2347</v>
+        <v>0.2301</v>
       </c>
       <c r="H11" t="inlineStr" s="3">
         <is>
@@ -1630,283 +1756,352 @@
         </is>
       </c>
       <c r="I11" s="4">
-        <v>0.2169</v>
+        <v>0.2457</v>
       </c>
       <c r="J11" t="inlineStr" s="3">
         <is>
-          <t>28/30</t>
+          <t>27/30</t>
         </is>
       </c>
       <c r="K11" s="4">
-        <v>0.6665</v>
+        <v>0.6963</v>
       </c>
       <c r="L11" s="4">
-        <v>0.5033</v>
+        <v>0.4581</v>
       </c>
       <c r="M11" s="3">
         <v>170.3863</v>
       </c>
       <c r="N11" s="3">
-        <v>174.21</v>
+        <v>177.92</v>
       </c>
       <c r="O11" s="3">
-        <v>4.36</v>
+        <v>4.943</v>
       </c>
       <c r="P11" t="inlineStr" s="3">
         <is>
-          <t>VENCEDOR ABSOLUTO DENTRO DO K=7 em Relevancy (0.2347), Correctness (0.2169) e Recall (0.5033)! Como seus chunks têm ~385 chars em média, eles cabem inteiros dentro do teto de 857 chars/chunk sem sofrer truncamento em K=7.</t>
+          <t>Salto expressivo em Faithfulness (+25.7%, de 0.3702 em K=3 para 0.4652 em K=5) e lidera o Context Recall dentro de K=5 (0.4581), pois 5 micro-chunks semânticos formam um contexto mais completo sem sofrer corte no limite de 1200 chars.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1">
       <c r="A12" t="inlineStr" s="3">
         <is>
+          <t>FIXED (K=7)</t>
+        </is>
+      </c>
+      <c r="B12" s="3">
+        <v>7</v>
+      </c>
+      <c r="C12" t="inlineStr" s="3">
+        <is>
+          <t>512 tokens | overlap 51 | teto 857 chars/chunk (TRUNCADO!)</t>
+        </is>
+      </c>
+      <c r="D12" s="3">
+        <v>207</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0.2693</v>
+      </c>
+      <c r="F12" t="inlineStr" s="3">
+        <is>
+          <t>28/30</t>
+        </is>
+      </c>
+      <c r="G12" s="4">
+        <v>0.1678</v>
+      </c>
+      <c r="H12" t="inlineStr" s="3">
+        <is>
+          <t>30/30</t>
+        </is>
+      </c>
+      <c r="I12" s="4">
+        <v>0.1728</v>
+      </c>
+      <c r="J12" t="inlineStr" s="3">
+        <is>
+          <t>26/30</t>
+        </is>
+      </c>
+      <c r="K12" s="4">
+        <v>0.7199</v>
+      </c>
+      <c r="L12" s="4">
+        <v>0.4022</v>
+      </c>
+      <c r="M12" s="4">
+        <v>0.0628</v>
+      </c>
+      <c r="N12" s="3">
+        <v>173.29</v>
+      </c>
+      <c r="O12" s="3">
+        <v>2.38</v>
+      </c>
+      <c r="P12" t="inlineStr" s="3">
+        <is>
+          <t>Queda acentuada em K=7: como RAG_MAX_CONTEXT_CHARS=6000 divide o orçamento por K (6000 // 7 = 857 chars/chunk), cada chunk Fixed (~1454 chars) perde ~41% do seu texto final! Além disso, mais chunks periféricos diluem a atenção do LLM (Lost in the Middle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" t="inlineStr" s="3">
+        <is>
+          <t>RECURSIVE (K=7)</t>
+        </is>
+      </c>
+      <c r="B13" s="3">
+        <v>7</v>
+      </c>
+      <c r="C13" t="inlineStr" s="3">
+        <is>
+          <t>512 tokens | overlap 51 | teto 857 chars/chunk (TRUNCADO!)</t>
+        </is>
+      </c>
+      <c r="D13" s="3">
+        <v>213</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0.3735</v>
+      </c>
+      <c r="F13" t="inlineStr" s="3">
+        <is>
+          <t>29/30</t>
+        </is>
+      </c>
+      <c r="G13" s="4">
+        <v>0.1647</v>
+      </c>
+      <c r="H13" t="inlineStr" s="3">
+        <is>
+          <t>30/30</t>
+        </is>
+      </c>
+      <c r="I13" s="4">
+        <v>0.1653</v>
+      </c>
+      <c r="J13" t="inlineStr" s="3">
+        <is>
+          <t>27/30</t>
+        </is>
+      </c>
+      <c r="K13" s="4">
+        <v>0.7187</v>
+      </c>
+      <c r="L13" s="4">
+        <v>0.4961</v>
+      </c>
+      <c r="M13" s="4">
+        <v>0.2182</v>
+      </c>
+      <c r="N13" s="3">
+        <v>175.61</v>
+      </c>
+      <c r="O13" s="3">
+        <v>3.127</v>
+      </c>
+      <c r="P13" t="inlineStr" s="3">
+        <is>
+          <t>O Context Recall subiu para 0.4961 (mais trechos do gabarito entraram nos 7 chunks), mas a qualidade da resposta (Relevancy 0.1647 / Correctness 0.1653) caiu pelo truncamento de 857 chars/chunk no gerador e pelo excesso de ruído no prompt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" t="inlineStr" s="3">
+        <is>
+          <t>SEMANTIC p60 (K=7)</t>
+        </is>
+      </c>
+      <c r="B14" s="3">
+        <v>7</v>
+      </c>
+      <c r="C14" t="inlineStr" s="3">
+        <is>
+          <t>Percentil 60 (p60) | teto 857 chars/chunk</t>
+        </is>
+      </c>
+      <c r="D14" s="3">
+        <v>781</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0.3481</v>
+      </c>
+      <c r="F14" t="inlineStr" s="3">
+        <is>
+          <t>26/30</t>
+        </is>
+      </c>
+      <c r="G14" s="4">
+        <v>0.2347</v>
+      </c>
+      <c r="H14" t="inlineStr" s="3">
+        <is>
+          <t>30/30</t>
+        </is>
+      </c>
+      <c r="I14" s="4">
+        <v>0.2169</v>
+      </c>
+      <c r="J14" t="inlineStr" s="3">
+        <is>
+          <t>28/30</t>
+        </is>
+      </c>
+      <c r="K14" s="4">
+        <v>0.6665</v>
+      </c>
+      <c r="L14" s="4">
+        <v>0.5033</v>
+      </c>
+      <c r="M14" s="3">
+        <v>170.3863</v>
+      </c>
+      <c r="N14" s="3">
+        <v>174.21</v>
+      </c>
+      <c r="O14" s="3">
+        <v>4.36</v>
+      </c>
+      <c r="P14" t="inlineStr" s="3">
+        <is>
+          <t>VENCEDOR ABSOLUTO DENTRO DO K=7 em Relevancy (0.2347), Correctness (0.2169) e Recall (0.5033)! Como seus chunks têm ~385 chars em média, eles cabem inteiros dentro do teto de 857 chars/chunk sem sofrer truncamento em K=7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" t="inlineStr" s="3">
+        <is>
           <t>BASELINE (Sem RAG)</t>
         </is>
       </c>
-      <c r="B12" s="3">
+      <c r="B15" s="3">
         <v>0</v>
       </c>
-      <c r="C12" t="inlineStr" s="3">
+      <c r="C15" t="inlineStr" s="3">
         <is>
           <t>Sem chunking e sem busca vetorial (contexts = [])</t>
         </is>
       </c>
-      <c r="D12" s="3">
+      <c r="D15" s="3">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr" s="3">
+      <c r="E15" t="inlineStr" s="3">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr" s="3">
+      <c r="F15" t="inlineStr" s="3">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="4">
+      <c r="G15" s="4">
         <v>0.1639</v>
       </c>
-      <c r="H12" t="inlineStr" s="3">
+      <c r="H15" t="inlineStr" s="3">
         <is>
           <t>30/30</t>
         </is>
       </c>
-      <c r="I12" s="4">
+      <c r="I15" s="4">
         <v>0.1467</v>
       </c>
-      <c r="J12" t="inlineStr" s="3">
+      <c r="J15" t="inlineStr" s="3">
         <is>
           <t>26/30</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr" s="3">
+      <c r="K15" t="inlineStr" s="3">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr" s="3">
+      <c r="L15" t="inlineStr" s="3">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M12" s="4">
+      <c r="M15" s="4">
         <v>0.0</v>
       </c>
-      <c r="N12" s="4">
+      <c r="N15" s="4">
         <v>0.0</v>
       </c>
-      <c r="O12" t="inlineStr" s="3">
+      <c r="O15" t="inlineStr" s="3">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr" s="3">
+      <c r="P15" t="inlineStr" s="3">
         <is>
           <t>Linha de base sem RAG: acerta apenas 0.1467 (Correctness) e 0.1639 (Relevancy). O ponto ótimo do RAG (K=5) supera o Baseline em até +93% em Relevancy (Recursive K=5 = 0.3169) e +69% em Correctness (Recursive K=5 = 0.2475).</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" t="inlineStr" s="1">
+    <row r="16"/>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" t="inlineStr" s="1">
         <is>
           <t>TABELA DETALHADA DE TEMPOS DE EXECUÇÃO (Fase 1 — Medido em NVIDIA A100 + CPU BGE-M3 para 30 QAs nos 10 PDFs)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" t="inlineStr" s="2">
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" t="inlineStr" s="2">
         <is>
           <t>Estratégia</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr" s="2">
+      <c r="B18" t="inlineStr" s="2">
         <is>
           <t>TOP_K</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="2">
+      <c r="C18" t="inlineStr" s="2">
         <is>
           <t>Nº de Chunks</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr" s="2">
+      <c r="D18" t="inlineStr" s="2">
         <is>
           <t>Tempo de Chunking (s)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr" s="2">
+      <c r="E18" t="inlineStr" s="2">
         <is>
           <t>Tempo de Indexação Chroma (s)</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr" s="2">
+      <c r="F18" t="inlineStr" s="2">
         <is>
           <t>Tempo Busca Total 30 QAs (s)</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr" s="2">
+      <c r="G18" t="inlineStr" s="2">
         <is>
           <t>Tempo Busca Médio por Pergunta (ms)</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr" s="2">
+      <c r="H18" t="inlineStr" s="2">
         <is>
           <t>Tempo Geração LLM Total 30 QAs (s)</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr" s="2">
+      <c r="I18" t="inlineStr" s="2">
         <is>
           <t>Tempo Geração LLM Médio por Pergunta (s)</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr" s="2">
+      <c r="J18" t="inlineStr" s="2">
         <is>
           <t>Tempo Total de Consulta Médio (Busca + LLM) (s/QA)</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr" s="2">
+      <c r="K18" t="inlineStr" s="2">
         <is>
           <t>Conclusão de Desempenho Operacional</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="44" customHeight="1">
-      <c r="A16" t="inlineStr" s="3">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="B16" s="3">
-        <v>5</v>
-      </c>
-      <c r="C16" s="3">
-        <v>207</v>
-      </c>
-      <c r="D16" s="4">
-        <v>0.0628</v>
-      </c>
-      <c r="E16" s="3">
-        <v>126.0329</v>
-      </c>
-      <c r="F16" s="3">
-        <v>5.5767</v>
-      </c>
-      <c r="G16" s="3">
-        <v>185.89</v>
-      </c>
-      <c r="H16" s="3">
-        <v>103.6991</v>
-      </c>
-      <c r="I16" s="3">
-        <v>3.457</v>
-      </c>
-      <c r="J16" s="3">
-        <v>3.643</v>
-      </c>
-      <c r="K16" t="inlineStr" s="3">
-        <is>
-          <t>Chunking instantâneo (0.06s) e menor tempo de resposta em K=5 (3.64s/pergunta).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="A17" t="inlineStr" s="3">
-        <is>
-          <t>recursive</t>
-        </is>
-      </c>
-      <c r="B17" s="3">
-        <v>5</v>
-      </c>
-      <c r="C17" s="3">
-        <v>213</v>
-      </c>
-      <c r="D17" s="4">
-        <v>0.2182</v>
-      </c>
-      <c r="E17" s="3">
-        <v>122.616</v>
-      </c>
-      <c r="F17" s="3">
-        <v>5.4412</v>
-      </c>
-      <c r="G17" s="3">
-        <v>181.37</v>
-      </c>
-      <c r="H17" s="3">
-        <v>131.9528</v>
-      </c>
-      <c r="I17" s="3">
-        <v>4.398</v>
-      </c>
-      <c r="J17" s="3">
-        <v>4.58</v>
-      </c>
-      <c r="K17" t="inlineStr" s="3">
-        <is>
-          <t>Melhor equilíbrio geral: chunking em 0.22s, busca em 181ms e melhor qualidade de resposta (Relevancy 0.3169 / Correctness 0.2475).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="44" customHeight="1">
-      <c r="A18" t="inlineStr" s="3">
-        <is>
-          <t>semantic (p60)</t>
-        </is>
-      </c>
-      <c r="B18" s="3">
-        <v>5</v>
-      </c>
-      <c r="C18" s="3">
-        <v>781</v>
-      </c>
-      <c r="D18" s="3">
-        <v>170.3863</v>
-      </c>
-      <c r="E18" s="3">
-        <v>131.6885</v>
-      </c>
-      <c r="F18" s="3">
-        <v>5.3376</v>
-      </c>
-      <c r="G18" s="3">
-        <v>177.92</v>
-      </c>
-      <c r="H18" s="3">
-        <v>148.299</v>
-      </c>
-      <c r="I18" s="3">
-        <v>4.943</v>
-      </c>
-      <c r="J18" s="3">
-        <v>5.121</v>
-      </c>
-      <c r="K18" t="inlineStr" s="3">
-        <is>
-          <t>Busca vetorial no Chroma continua rápida (177.9ms mesmo com 781 chunks), mas o chunking leva 170.39s (~2.700x mais lento que Fixed) e a geração LLM leva 4.94s/pergunta.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +2112,7 @@
         </is>
       </c>
       <c r="B19" s="3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C19" s="3">
         <v>207</v>
@@ -1929,23 +2124,23 @@
         <v>126.0329</v>
       </c>
       <c r="F19" s="3">
-        <v>5.1987</v>
+        <v>5.5767</v>
       </c>
       <c r="G19" s="3">
-        <v>173.29</v>
+        <v>185.89</v>
       </c>
       <c r="H19" s="3">
-        <v>71.4038</v>
+        <v>103.6991</v>
       </c>
       <c r="I19" s="3">
-        <v>2.38</v>
+        <v>3.457</v>
       </c>
       <c r="J19" s="3">
-        <v>2.553</v>
+        <v>3.643</v>
       </c>
       <c r="K19" t="inlineStr" s="3">
         <is>
-          <t>Geração mais rápida em K=7 (2.38s/pergunta) porque o modelo se abstém com mais frequência ('Não encontrei no contexto') quando os chunks vêm truncados em 857 chars.</t>
+          <t>Chunking instantâneo (0.06s) e menor tempo de resposta em K=5 (3.64s/pergunta).</t>
         </is>
       </c>
     </row>
@@ -1956,7 +2151,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C20" s="3">
         <v>213</v>
@@ -1968,23 +2163,23 @@
         <v>122.616</v>
       </c>
       <c r="F20" s="3">
-        <v>5.2682</v>
+        <v>5.4412</v>
       </c>
       <c r="G20" s="3">
-        <v>175.61</v>
+        <v>181.37</v>
       </c>
       <c r="H20" s="3">
-        <v>93.8097</v>
+        <v>131.9528</v>
       </c>
       <c r="I20" s="3">
-        <v>3.127</v>
+        <v>4.398</v>
       </c>
       <c r="J20" s="3">
-        <v>3.303</v>
+        <v>4.58</v>
       </c>
       <c r="K20" t="inlineStr" s="3">
         <is>
-          <t>Busca em 175.6ms e geração em 3.13s/pergunta (respostas mais curtas/abstêmias devido ao truncamento por chunk em K=7).</t>
+          <t>Melhor equilíbrio geral: chunking em 0.22s, busca em 181ms e melhor qualidade de resposta (Relevancy 0.3169 / Correctness 0.2475).</t>
         </is>
       </c>
     </row>
@@ -1995,7 +2190,7 @@
         </is>
       </c>
       <c r="B21" s="3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C21" s="3">
         <v>781</v>
@@ -2007,97 +2202,214 @@
         <v>131.6885</v>
       </c>
       <c r="F21" s="3">
+        <v>5.3376</v>
+      </c>
+      <c r="G21" s="3">
+        <v>177.92</v>
+      </c>
+      <c r="H21" s="3">
+        <v>148.299</v>
+      </c>
+      <c r="I21" s="3">
+        <v>4.943</v>
+      </c>
+      <c r="J21" s="3">
+        <v>5.121</v>
+      </c>
+      <c r="K21" t="inlineStr" s="3">
+        <is>
+          <t>Busca vetorial no Chroma continua rápida (177.9ms mesmo com 781 chunks), mas o chunking leva 170.39s (~2.700x mais lento que Fixed) e a geração LLM leva 4.94s/pergunta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="A22" t="inlineStr" s="3">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="B22" s="3">
+        <v>7</v>
+      </c>
+      <c r="C22" s="3">
+        <v>207</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0.0628</v>
+      </c>
+      <c r="E22" s="3">
+        <v>126.0329</v>
+      </c>
+      <c r="F22" s="3">
+        <v>5.1987</v>
+      </c>
+      <c r="G22" s="3">
+        <v>173.29</v>
+      </c>
+      <c r="H22" s="3">
+        <v>71.4038</v>
+      </c>
+      <c r="I22" s="3">
+        <v>2.38</v>
+      </c>
+      <c r="J22" s="3">
+        <v>2.553</v>
+      </c>
+      <c r="K22" t="inlineStr" s="3">
+        <is>
+          <t>Geração mais rápida em K=7 (2.38s/pergunta) porque o modelo se abstém com mais frequência ('Não encontrei no contexto') quando os chunks vêm truncados em 857 chars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
+      <c r="A23" t="inlineStr" s="3">
+        <is>
+          <t>recursive</t>
+        </is>
+      </c>
+      <c r="B23" s="3">
+        <v>7</v>
+      </c>
+      <c r="C23" s="3">
+        <v>213</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0.2182</v>
+      </c>
+      <c r="E23" s="3">
+        <v>122.616</v>
+      </c>
+      <c r="F23" s="3">
+        <v>5.2682</v>
+      </c>
+      <c r="G23" s="3">
+        <v>175.61</v>
+      </c>
+      <c r="H23" s="3">
+        <v>93.8097</v>
+      </c>
+      <c r="I23" s="3">
+        <v>3.127</v>
+      </c>
+      <c r="J23" s="3">
+        <v>3.303</v>
+      </c>
+      <c r="K23" t="inlineStr" s="3">
+        <is>
+          <t>Busca em 175.6ms e geração em 3.13s/pergunta (respostas mais curtas/abstêmias devido ao truncamento por chunk em K=7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
+      <c r="A24" t="inlineStr" s="3">
+        <is>
+          <t>semantic (p60)</t>
+        </is>
+      </c>
+      <c r="B24" s="3">
+        <v>7</v>
+      </c>
+      <c r="C24" s="3">
+        <v>781</v>
+      </c>
+      <c r="D24" s="3">
+        <v>170.3863</v>
+      </c>
+      <c r="E24" s="3">
+        <v>131.6885</v>
+      </c>
+      <c r="F24" s="3">
         <v>5.2263</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G24" s="3">
         <v>174.21</v>
       </c>
-      <c r="H21" s="3">
+      <c r="H24" s="3">
         <v>130.8042</v>
       </c>
-      <c r="I21" s="3">
+      <c r="I24" s="3">
         <v>4.36</v>
       </c>
-      <c r="J21" s="3">
+      <c r="J24" s="3">
         <v>4.534</v>
       </c>
-      <c r="K21" t="inlineStr" s="3">
+      <c r="K24" t="inlineStr" s="3">
         <is>
           <t>Mantém respostas completas em K=7 (4.36s/pergunta) porque seus chunks (~385 chars) não sofrem corte no teto de 857 chars.</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" t="inlineStr" s="1">
+    <row r="25"/>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" t="inlineStr" s="1">
         <is>
           <t>SÍNTESE DOS ACHADOS DA CURVA DE TOP_K (K=3 vs K=5 vs K=7) PARA A REDAÇÃO DO TCC</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" t="inlineStr" s="2">
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" t="inlineStr" s="2">
         <is>
           <t>Achado Científico</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr" s="2">
+      <c r="B27" t="inlineStr" s="2">
         <is>
           <t>Evidência Experimental nos Dados</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr" s="2">
+      <c r="C27" t="inlineStr" s="2">
         <is>
           <t>Interpretação para o TCC</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="44" customHeight="1">
-      <c r="A25" t="inlineStr" s="3">
+    <row r="28" ht="44" customHeight="1">
+      <c r="A28" t="inlineStr" s="3">
         <is>
           <t>1. O Ponto Ótimo da Curva é TOP_K = 5</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr" s="3">
+      <c r="B28" t="inlineStr" s="3">
         <is>
           <t>Ao subir de K=3 para K=5: Faithfulness saltou em Fixed (0.4002 -&gt; 0.4882, +22%) e Semantic (0.3702 -&gt; 0.4652, +25.7%); Answer Relevancy e Answer Correctness do Recursive saltaram +46% (0.2173 -&gt; 0.3169) e +18% (0.2098 -&gt; 0.2475).</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr" s="3">
+      <c r="C28" t="inlineStr" s="3">
         <is>
           <t>Em um corpus de 10 documentos onde perguntas de Nível 2 e Nível 3 exigem cruzar de 2 a 6 PDFs, K=3 é insuficiente para cobrir todas as fontes. Já K=5 fornece cobertura multi-documento sem saturar o prompt.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="44" customHeight="1">
-      <c r="A26" t="inlineStr" s="3">
+    <row r="29" ht="44" customHeight="1">
+      <c r="A29" t="inlineStr" s="3">
         <is>
           <t>2. Saturação e Degradação em TOP_K = 7</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr" s="3">
+      <c r="B29" t="inlineStr" s="3">
         <is>
           <t>Ao subir de K=5 para K=7: todas as métricas de geração caíram (Faithfulness caiu para 0.2693-0.3735; Correctness caiu para 0.1653-0.2169), embora o Context Recall tenha subido para ~0.50 no Recursive (0.4961) e Semantic (0.5033).</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr" s="3">
+      <c r="C29" t="inlineStr" s="3">
         <is>
           <t>Comprova dois fenômenos clássicos da literatura de RAG: (a) 'Lost in the Middle' / diluição de atenção (entregar 7 trechos inclui chunks de menor similaridade que confundem o LLM de 8B parâmetros) e (b) competição pelo orçamento de contexto (RAG_MAX_CONTEXT_CHARS = 6000 chars dividido por 7 reduz o teto por chunk para 857 chars, truncando chunks de 512 tokens).</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="44" customHeight="1">
-      <c r="A27" t="inlineStr" s="3">
+    <row r="30" ht="44" customHeight="1">
+      <c r="A30" t="inlineStr" s="3">
         <is>
           <t>3. Trade-off Custo Computacional vs. Granularidade Semântica</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr" s="3">
+      <c r="B30" t="inlineStr" s="3">
         <is>
           <t>O Semantic Chunker (p60) demora 170.39s para segmentar os 10 PDFs (contra 0.06s do Fixed e 0.22s do Recursive), mas é o mais resiliente em K=7 (Correctness 0.2169 vs 0.1653 do Recursive) e líder em Context Recall (0.5085 em K=3, 0.4581 em K=5, 0.5033 em K=7).</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr" s="3">
+      <c r="C30" t="inlineStr" s="3">
         <is>
           <t>O Semantic Chunker cria blocos menores e tematicamente puros (~385 chars), o que maximiza a revocação (Recall) em múltiplos documentos e evita truncamento em K alto, mas a um custo de pré-processamento 780x maior que o Recursive. O Recursive em K=5 entrega a maior corretude (0.2475) e relevância (0.3169) com custo de chunking desprezível (0.22s).</t>
         </is>

</xml_diff>